<commit_message>
CharacterTable 스킬1/2/3 정보 최신화 (v0.5.3)
인격 스킬명/속성/유형/아이콘을 최신 데이터로 갱신. 181개 인격 전체 스킬1~3
정보 확인 완료 (아이콘 일부 누락은 원본 데이터 기준).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/UpdateLog.xlsx
+++ b/UpdateLog.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C23"/>
+  <dimension ref="A1:C24"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -668,9 +668,20 @@
         <v>정답 공개, 스킬 퀴즈, 결과 카드에서 각성 이미지를 기본으로 표시하도록 변경 (각성 이미지가 없으면 일반 이미지로 대체)</v>
       </c>
     </row>
+    <row r="24">
+      <c r="A24" t="str">
+        <v>v0.5.3</v>
+      </c>
+      <c r="B24" t="str">
+        <v>2026-07-02</v>
+      </c>
+      <c r="C24" t="str">
+        <v>CharacterTable.xlsx 스킬1/2/3 정보(명칭·속성·유형·아이콘) 최신화 반영</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C23"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C24"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
CharacterTable에 ID열 추가 (v0.13.18)
인격 고유 번호를 A열(ID)로 노출하고 build-data.js에도 반영해
data.json에서 바로 참조할 수 있도록 함.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/UpdateLog.xlsx
+++ b/UpdateLog.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C59"/>
+  <dimension ref="A1:C60"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1129,9 +1129,21 @@
 외부 CDN 대신 프로젝트 내 이미지를 사용해 로딩 안정성 향상</v>
       </c>
     </row>
+    <row r="60" xml:space="preserve">
+      <c r="A60" t="str">
+        <v>v0.13.18</v>
+      </c>
+      <c r="B60" t="str">
+        <v>2026-07-08</v>
+      </c>
+      <c r="C60" t="str" xml:space="preserve">
+        <v xml:space="preserve">CharacterTable에 ID열(A열) 추가
+인격 고유 번호를 데이터에 노출해 추후 참조/매칭에 사용할 수 있도록 함</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C59"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C60"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
changelog_dev.json이 실제로 공개 배포되던 문제 수정 (v0.13.30)
.vercelignore는 배포 업로드 시점의 소스 파일 필터일 뿐, 빌드 명령
실행 중에 새로 생성되는 파일에는 적용되지 않는다는 것을 확인했다.
outputDirectory가 "."이라 dev/changelog_dev.json이 빌드 후 그대로
공개 URL로 서빙되고 있었음(실제 배포 사이트에서 200 OK로 확인).

수정: Vercel 빌드 환경(자동 설정되는 VERCEL=1)에서는 changelog_dev.json
자체를 생성하지 않도록 해서 배포 산출물에 아예 포함되지 않게 했다.
로컬 개발 환경에서는 기존처럼 dev/changelog_dev.json이 정상 생성된다.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/UpdateLog.xlsx
+++ b/UpdateLog.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D71"/>
+  <dimension ref="A1:D72"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1495,9 +1495,24 @@
         <v/>
       </c>
     </row>
+    <row r="72" xml:space="preserve">
+      <c r="A72" t="str">
+        <v>v0.13.30</v>
+      </c>
+      <c r="B72" t="str">
+        <v>2026-07-10</v>
+      </c>
+      <c r="C72" t="str" xml:space="preserve">
+        <v xml:space="preserve">.vercelignore는 빌드 중 새로 생성되는 파일에는 적용되지 않아 changelog_dev.json이 실제로는 공개 배포되고 있던 것을 발견하고 수정
+Vercel 빌드 환경(VERCEL=1)에서는 changelog_dev.json 자체를 생성하지 않도록 변경, 로컬에서는 그대로 생성됨</v>
+      </c>
+      <c r="D72" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D71"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D72"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
v0.13.66: 신규 인격 'LCE E.G.O::차원찢개 이상'(10116) 추가
- CharacterData/SkillData에 10116 등록, 인격/각성/스킬1-3 이미지 5종 추가
- CharacterTable의 이미지(일반) 경로 오타 수정
  (10116_nromal.png → 10116_normal.png)

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/UpdateLog.xlsx
+++ b/UpdateLog.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\imtl\limquiz\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BC8322B2-0EC8-48A1-ADC9-D0CD19A0E3F4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{992D84E3-3CB2-4CE4-96B1-2B5D61EAAB65}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28770" yWindow="0" windowWidth="28830" windowHeight="15600" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="UpdateLog" sheetId="1" r:id="rId1"/>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="638" uniqueCount="316">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="642" uniqueCount="320">
   <si>
     <t>버전</t>
   </si>
@@ -1206,6 +1206,20 @@
   <si>
     <t>스킬 퀴즈: 제출·힌트 사용 횟수 표시가 스티키 정보 영역 안으로 들어가 스크롤해도 계속 보입니다.
 스킬 퀴즈: 이름 힌트를 여러 번 눌러도 처음 봤던 글자 수 안내가 사라지지 않고, 글자 공개 힌트만 갱신됩니다.</t>
+  </si>
+  <si>
+    <t>v0.13.66</t>
+  </si>
+  <si>
+    <t>2026-07-22</t>
+  </si>
+  <si>
+    <t>신규 인격 10116(LCE E.G.O::차원찢개 이상) 추가: CharacterData/SkillData 행 확인, 이미지(일반) 경로 오타 수정(10116_nromal.png → 10116_normal.png, 실제 파일명과 불일치했음). 인격/각성/스킬1-3 이미지 5종 로컬 커밋. slug-map.json에는 항목 미추가(CDN 슬러그 추측 시 깨진 링크 위험, 로컬 이미지가 있어 게임 플레이엔 영향 없음 - 빌드가 "slug 없음" 경고만 냄)
+data.json 184개 인격으로 재생성, 신규 인격 필드 전부 정상(스킬명/속성/유형/아이콘, 키워드, 이미지 경로) 확인
+검증: 이미지 5종 fetch 200, DATA에서 인격 조회 성공</t>
+  </si>
+  <si>
+    <t>신규 인격 'LCE E.G.O::차원찢개 이상'이 추가되었습니다.</t>
   </si>
 </sst>
 </file>
@@ -1593,7 +1607,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D107"/>
+  <dimension ref="A1:D108"/>
   <sheetFormatPr defaultRowHeight="17.25" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.3">
@@ -3092,6 +3106,20 @@
       </c>
       <c r="D107" s="2" t="s">
         <v>315</v>
+      </c>
+    </row>
+    <row r="108" spans="1:4" ht="409.5" x14ac:dyDescent="0.3">
+      <c r="A108" t="s">
+        <v>316</v>
+      </c>
+      <c r="B108" s="1" t="s">
+        <v>317</v>
+      </c>
+      <c r="C108" s="2" t="s">
+        <v>318</v>
+      </c>
+      <c r="D108" s="2" t="s">
+        <v>319</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add random EGO Wordle mode
</commit_message>
<xml_diff>
--- a/UpdateLog.xlsx
+++ b/UpdateLog.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="UpdateLog" sheetId="1" r:id="R7490b6adfbdd46fe"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="UpdateLog_백업" sheetId="2" r:id="R074a441141b447b2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="UpdateLog" sheetId="1" r:id="R0d5e20f283294ee8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="UpdateLog_백업" sheetId="2" r:id="R011a78f03d204949"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -3308,6 +3308,26 @@
 모바일 상단 버튼이 화면 밖으로 잘리던 문제와 게임 화면 이동 시 이전 스크롤 위치가 남던 문제를 수정했습니다.</x:v>
       </x:c>
     </x:row>
+    <x:row r="126">
+      <x:c r="A126" t="str">
+        <x:v>v0.14.1</x:v>
+      </x:c>
+      <x:c r="B126" t="str">
+        <x:v>2026-08-27</x:v>
+      </x:c>
+      <x:c r="C126" t="str">
+        <x:v>홈 화면에 EGO 랜덤 플레이 진입 카드 추가
+오늘의 EGO와 랜덤 모드가 동일한 6칸 비교 판정 및 6회 제한 엔진을 공유하도록 구조 확장
+랜덤 모드 결과에 다음 랜덤 EGO 버튼을 추가하고 직전 정답 연속 출제 방지
+랜덤 진행·결과를 일일 localStorage 상태와 28일 활동 잔디에서 분리
+EGO 랜덤 플레이 기록과 스포일러 방지 판정 격자 공유 카드 지원</x:v>
+      </x:c>
+      <x:c r="D126" t="str">
+        <x:v>홈에 EGO 랜덤 플레이가 추가되었습니다. 무작위 EGO를 6번 안에 맞히고, 결과 화면에서 바로 다음 문제에 계속 도전할 수 있습니다.
+랜덤 플레이도 오늘의 EGO와 같은 비교 판정을 사용하며 같은 EGO가 연속으로 출제되지 않습니다.
+랜덤 플레이 기록은 저장되지만 오늘의 EGO 진행 상황과 최근 28일 일일 활동에는 영향을 주지 않습니다.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>

<commit_message>
Rework EGO Gift quiz and home navigation
</commit_message>
<xml_diff>
--- a/UpdateLog.xlsx
+++ b/UpdateLog.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="UpdateLog" sheetId="1" r:id="R0d5e20f283294ee8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="UpdateLog_백업" sheetId="2" r:id="R011a78f03d204949"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="UpdateLog" sheetId="1" r:id="Rfbbc704c0a8e456b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="UpdateLog_백업" sheetId="2" r:id="Re8370cee185b4554"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -3328,6 +3328,26 @@
 랜덤 플레이 기록은 저장되지만 오늘의 EGO 진행 상황과 최근 28일 일일 활동에는 영향을 주지 않습니다.</x:v>
       </x:c>
     </x:row>
+    <x:row r="127">
+      <x:c r="A127" t="str">
+        <x:v>v0.15.0</x:v>
+      </x:c>
+      <x:c r="B127" t="str">
+        <x:v>2026-08-28</x:v>
+      </x:c>
+      <x:c r="C127" t="str">
+        <x:v>• EGO 기프트에 날짜 시드 일일 답안, 진행 복원, 일일 결과 중복 방지와 랜덤 연속 출제를 구현.
+• GQ 비교 필드 6종(등급 방향, 죄악 속성, 이름 길이 방향, 효과 줄 수 방향, 키워드 수 방향, 공통 키워드) 및 스포일러 없는 공유 카드를 추가.
+• EGO/GQ 판정 셀 순차 3D 플립, 라운드 진입, 결과 패널 스태거를 추가하고 reduce-motion 설정을 유지.
+• 홈을 TODAY'S DIRECTIVES / TRAINING ARCHIVE / TACTICAL EXAMS로 재배치하고 일일 활동을 인격·EGO·기프트 3종 기준으로 확장.
+• 데스크톱·390px 모바일, 일일 오답/복원/정답, 랜덤 다음 문제, 콘솔 오류 없음까지 브라우저 검증.</x:v>
+      </x:c>
+      <x:c r="D127" t="str">
+        <x:v>• EGO 기프트 퀴즈를 오늘의 문제와 랜덤 훈련으로 분리했습니다.
+• 6번의 추측 동안 등급·속성·이름 길이·효과 줄·키워드 정보를 비교합니다.
+• EGO와 기프트 판정 애니메이션을 개선하고 홈 모드를 세 그룹으로 정리했습니다.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>

<commit_message>
Add v0.15.1 update log
</commit_message>
<xml_diff>
--- a/UpdateLog.xlsx
+++ b/UpdateLog.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="UpdateLog" sheetId="1" r:id="Rfbbc704c0a8e456b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="UpdateLog_백업" sheetId="2" r:id="Re8370cee185b4554"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="UpdateLog" sheetId="1" r:id="R1f18fd0096d24b16"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="UpdateLog_백업" sheetId="2" r:id="R80ec4d8ff1a54ed4"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -3348,6 +3348,26 @@
 • EGO와 기프트 판정 애니메이션을 개선하고 홈 모드를 세 그룹으로 정리했습니다.</x:v>
       </x:c>
     </x:row>
+    <x:row r="128">
+      <x:c r="A128" t="str">
+        <x:v>v0.15.1</x:v>
+      </x:c>
+      <x:c r="B128" t="str">
+        <x:v>2026-08-28</x:v>
+      </x:c>
+      <x:c r="C128" t="str">
+        <x:v>EGO 기프트 원본 keywordName을 데이터 파이프라인에 추가하고, 범용은 키워드 없음으로 정규화.
+기프트 효과 문장에 등장하는 상태이상 개수 추정 대신 실제 단일 키워드의 정확 일치 판정으로 변경.
+모든 기프트에 붙는 내부 attrKeywordId와 실제 효과 조건을 분리하고, 공명·속성 스킬 조건에서 조건속성을 계산하도록 구현.
+속성 조건 없음 및 복수 속성 조건을 지원하고, 속성 묶음이 정확히 같을 때만 일치하도록 GQ 비교·결과 UI 수정.
+검증: 기프트 441개, 키워드 없음 109개, 속성 조건 없음 361개, 복수 속성 조건 7개.</x:v>
+      </x:c>
+      <x:c r="D128" t="str">
+        <x:v>EGO 기프트 퀴즈의 키워드와 속성 판정을 수정했습니다.
+키워드는 실제 기프트 분류가 정확히 같을 때만 일치합니다.
+속성은 공명·속성 스킬로 추가 효과가 발동하는 조건만 비교하며, 조건이 없거나 여러 개인 기프트도 정확하게 표시됩니다.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>

<commit_message>
Add progressive EGO gift effect clues
</commit_message>
<xml_diff>
--- a/UpdateLog.xlsx
+++ b/UpdateLog.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="UpdateLog" sheetId="1" r:id="R1f18fd0096d24b16"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="UpdateLog_백업" sheetId="2" r:id="R80ec4d8ff1a54ed4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="UpdateLog" sheetId="1" r:id="R908da96c949f4fe6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="UpdateLog_백업" sheetId="2" r:id="Rd0a6946882a34d45"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -3368,6 +3368,27 @@
 속성은 공명·속성 스킬로 추가 효과가 발동하는 조건만 비교하며, 조건이 없거나 여러 개인 기프트도 정확하게 표시됩니다.</x:v>
       </x:c>
     </x:row>
+    <x:row r="129">
+      <x:c r="A129" t="str">
+        <x:v>v0.15.2</x:v>
+      </x:c>
+      <x:c r="B129" t="str">
+        <x:v>2026-08-28</x:v>
+      </x:c>
+      <x:c r="C129" t="str">
+        <x:v>EGO 기프트 퀴즈의 효과 줄 수 비교를 제거하고, 원본 enhanceYn 기반 강화 가능 여부 판정으로 교체.
+강화 가능 기프트 ID 116개를 별도 데이터로 생성하고 빌드 파이프라인에서 각 기프트의 강화가능 필드를 구성.
+효과 설명을 문장·구절 기준 최대 6개 기록으로 나눠 첫 단서를 즉시 공개하고, 오답마다 다음 단서가 열리도록 구현.
+정답 키워드와 조건속성은 효과 문장 안에서 가리고, 해당 비교 판정이 정확히 일치한 뒤에만 원문을 해금.
+기존 일일 진행 복원·랜덤 모드·결과 공유와 호환되며 공유 요약의 효과 줄 항목을 강화 가능 여부로 변경.
+데스크톱 및 390px 모바일 렌더, 가로 넘침 없음, HTML 스크립트 파싱과 기프트 441개 재빌드 검증.</x:v>
+      </x:c>
+      <x:c r="D129" t="str">
+        <x:v>EGO 기프트 퀴즈에서 효과 줄 수 비교를 없애고 강화 가능 여부로 바꿨습니다.
+효과 기록의 첫 단서는 처음부터 보이며, 오답을 낼 때마다 다음 효과 단서가 하나씩 열립니다.
+효과 문장 속 키워드와 조건 속성은 처음에는 가려지고, 관련 판정을 정확히 맞히면 해금됩니다.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>

<commit_message>
Move EGO answers above guess history
</commit_message>
<xml_diff>
--- a/UpdateLog.xlsx
+++ b/UpdateLog.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="UpdateLog" sheetId="1" r:id="R908da96c949f4fe6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="UpdateLog_백업" sheetId="2" r:id="Rd0a6946882a34d45"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="UpdateLog" sheetId="1" r:id="R590d369223504e40"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="UpdateLog_백업" sheetId="2" r:id="Ra4479cc3498c4be5"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -3389,6 +3389,22 @@
 효과 문장 속 키워드와 조건 속성은 처음에는 가려지고, 관련 판정을 정확히 맞히면 해금됩니다.</x:v>
       </x:c>
     </x:row>
+    <x:row r="130">
+      <x:c r="A130" t="str">
+        <x:v>v0.15.3</x:v>
+      </x:c>
+      <x:c r="B130" t="str">
+        <x:v>2026-08-28</x:v>
+      </x:c>
+      <x:c r="C130" t="str">
+        <x:v>EGO 및 EGO 기프트 결과 화면의 DOM 순서를 조정해 정답 상세 패널(정보·효과·이미지)을 추측 판정 기록보다 먼저 렌더링.
+일일·랜덤 결과 렌더러에 공통 적용하고 결과 저장·공유·다음 문제 동작은 유지.
+데스크톱과 390px 모바일에서 정답 패널이 추측 기록보다 위에 위치하고 가로 넘침이 없음을 브라우저 검증.</x:v>
+      </x:c>
+      <x:c r="D130" t="str">
+        <x:v>EGO와 EGO 기프트 결과 화면에서 정답 정보와 이미지가 추측 기록보다 먼저 보이도록 상단으로 옮겼습니다.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>